<commit_message>
added korsce rankings for evaluation
</commit_message>
<xml_diff>
--- a/code/results/results_consolidated_excel.xlsx
+++ b/code/results/results_consolidated_excel.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://tud365-my.sharepoint.com/personal/hrishitachakra_tudelft_nl/Documents/Documents/SOL/Projects/conferences/UMAP'26/ChildCenteredEvaluation/code/results/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="6" documentId="8_{283E06E4-DE93-4185-AC54-65FDA09D846A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{65BBD7CD-1148-455E-867D-4E6447588DFC}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{60EAE184-8A2C-4F63-974D-A5B9AE745BCA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="16680" yWindow="-16605" windowWidth="29040" windowHeight="15720" xr2:uid="{46A0C11A-E1A4-481F-A370-EA49784679F9}"/>
+    <workbookView xWindow="18870" yWindow="-14550" windowWidth="21600" windowHeight="11175" xr2:uid="{D2ED2519-EAFD-47DA-804C-EDB526E2FA84}"/>
   </bookViews>
   <sheets>
     <sheet name="results_consolidated" sheetId="1" r:id="rId1"/>
@@ -557,11 +557,8 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -936,7 +933,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1E46A536-C3E8-4DF9-B4B4-03C58F0E28F5}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2BDE53CD-3062-4565-A278-B5B6E69685EC}">
   <dimension ref="A1:O10"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
@@ -944,24 +941,12 @@
       <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1"/>
-      <c r="F1" s="1"/>
-      <c r="G1" s="1"/>
-      <c r="H1" s="1"/>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>2</v>
       </c>
-      <c r="J1" s="1"/>
-      <c r="K1" s="1"/>
-      <c r="L1" s="1"/>
-      <c r="M1" s="1"/>
-      <c r="N1" s="1"/>
-      <c r="O1" s="1"/>
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.35">
       <c r="B2" t="s">
@@ -1012,46 +997,46 @@
         <v>10</v>
       </c>
       <c r="B3">
-        <v>0.59899999999999998</v>
+        <v>0.59921539387600797</v>
       </c>
       <c r="C3">
-        <v>0.54</v>
+        <v>0.54030463180800004</v>
       </c>
       <c r="D3">
-        <v>0.76300000000000001</v>
+        <v>0.76338095238095205</v>
       </c>
       <c r="E3">
-        <v>0.49299999999999999</v>
+        <v>0.49304761904761801</v>
       </c>
       <c r="F3">
-        <v>0.19900000000000001</v>
+        <v>0.198888888888888</v>
       </c>
       <c r="G3">
-        <v>0.67100000000000004</v>
+        <v>0.671190476190476</v>
       </c>
       <c r="H3">
-        <v>6.5000000000000002E-2</v>
+        <v>6.4959500252944405E-2</v>
       </c>
       <c r="I3">
-        <v>0.32900000000000001</v>
+        <v>0.32935841185663201</v>
       </c>
       <c r="J3">
-        <v>7.1999999999999995E-2</v>
+        <v>7.2256971551219504E-2</v>
       </c>
       <c r="K3">
-        <v>0.27700000000000002</v>
+        <v>0.27727932636469199</v>
       </c>
       <c r="L3">
-        <v>0.214</v>
+        <v>0.21396631823460999</v>
       </c>
       <c r="M3">
-        <v>2E-3</v>
+        <v>2.0325203252032002E-3</v>
       </c>
       <c r="N3">
-        <v>0.185</v>
+        <v>0.185172280294231</v>
       </c>
       <c r="O3">
-        <v>8.0000000000000002E-3</v>
+        <v>8.0767436494131005E-3</v>
       </c>
     </row>
     <row r="4" spans="1:15" x14ac:dyDescent="0.35">
@@ -1059,46 +1044,46 @@
         <v>11</v>
       </c>
       <c r="B4">
-        <v>0.58699999999999997</v>
+        <v>0.587288640153112</v>
       </c>
       <c r="C4">
-        <v>0.53700000000000003</v>
+        <v>0.53684445798399905</v>
       </c>
       <c r="D4">
-        <v>0.74399999999999999</v>
+        <v>0.74385714285714299</v>
       </c>
       <c r="E4">
-        <v>0.46899999999999997</v>
+        <v>0.46919047619047599</v>
       </c>
       <c r="F4">
-        <v>0.19900000000000001</v>
+        <v>0.198888888888888</v>
       </c>
       <c r="G4">
         <v>0.67</v>
       </c>
       <c r="H4">
-        <v>6.5000000000000002E-2</v>
+        <v>6.50162399347404E-2</v>
       </c>
       <c r="I4">
-        <v>0.33</v>
+        <v>0.32953444699226297</v>
       </c>
       <c r="J4">
-        <v>7.1999999999999995E-2</v>
+        <v>7.2359271648780504E-2</v>
       </c>
       <c r="K4">
-        <v>0.27700000000000002</v>
+        <v>0.27744870305845898</v>
       </c>
       <c r="L4">
-        <v>0.214</v>
+        <v>0.214135694928377</v>
       </c>
       <c r="M4">
-        <v>2E-3</v>
+        <v>2.0325203252032002E-3</v>
       </c>
       <c r="N4">
-        <v>0.185</v>
+        <v>0.18534165698799801</v>
       </c>
       <c r="O4">
-        <v>8.0000000000000002E-3</v>
+        <v>8.0767436494131005E-3</v>
       </c>
     </row>
     <row r="5" spans="1:15" x14ac:dyDescent="0.35">
@@ -1106,46 +1091,46 @@
         <v>12</v>
       </c>
       <c r="B5">
-        <v>0.58299999999999996</v>
+        <v>0.58348328159684903</v>
       </c>
       <c r="C5">
-        <v>0.52700000000000002</v>
+        <v>0.527163547647999</v>
       </c>
       <c r="D5">
-        <v>0.80300000000000005</v>
+        <v>0.80288888888888799</v>
       </c>
       <c r="E5">
-        <v>0.47699999999999998</v>
+        <v>0.47655555555555501</v>
       </c>
       <c r="F5">
-        <v>0.2</v>
+        <v>0.200333333333333</v>
       </c>
       <c r="G5">
-        <v>0.67900000000000005</v>
+        <v>0.67883333333333296</v>
       </c>
       <c r="H5">
-        <v>6.4000000000000001E-2</v>
+        <v>6.4244729252830896E-2</v>
       </c>
       <c r="I5">
-        <v>0.35899999999999999</v>
+        <v>0.35924009192589601</v>
       </c>
       <c r="J5">
-        <v>7.9000000000000001E-2</v>
+        <v>7.8921518204878E-2</v>
       </c>
       <c r="K5">
-        <v>0.29599999999999999</v>
+        <v>0.29628339140534199</v>
       </c>
       <c r="L5">
-        <v>0.23400000000000001</v>
+        <v>0.23414150212930701</v>
       </c>
       <c r="M5">
-        <v>2E-3</v>
+        <v>1.7421602787455999E-3</v>
       </c>
       <c r="N5">
-        <v>0.20799999999999999</v>
+        <v>0.20751548586914401</v>
       </c>
       <c r="O5">
-        <v>8.9999999999999993E-3</v>
+        <v>8.8760916695388992E-3</v>
       </c>
     </row>
     <row r="6" spans="1:15" x14ac:dyDescent="0.35">
@@ -1153,46 +1138,46 @@
         <v>13</v>
       </c>
       <c r="B6">
-        <v>0.64300000000000002</v>
+        <v>0.64336930449459795</v>
       </c>
       <c r="C6">
-        <v>0.57199999999999995</v>
+        <v>0.57184008192000002</v>
       </c>
       <c r="D6">
-        <v>0.748</v>
+        <v>0.74816666666666598</v>
       </c>
       <c r="E6">
-        <v>0.496</v>
+        <v>0.49627777777777698</v>
       </c>
       <c r="F6">
-        <v>0.16200000000000001</v>
+        <v>0.16211111111111101</v>
       </c>
       <c r="G6">
-        <v>0.64400000000000002</v>
+        <v>0.64433333333333298</v>
       </c>
       <c r="H6">
-        <v>6.3E-2</v>
+        <v>6.3445627191335299E-2</v>
       </c>
       <c r="I6">
-        <v>0.34200000000000003</v>
+        <v>0.341833394105378</v>
       </c>
       <c r="J6">
-        <v>7.4999999999999997E-2</v>
+        <v>7.5461949190243904E-2</v>
       </c>
       <c r="K6">
-        <v>0.27800000000000002</v>
+        <v>0.277671312427409</v>
       </c>
       <c r="L6">
-        <v>0.23499999999999999</v>
+        <v>0.23549651567944199</v>
       </c>
       <c r="M6">
-        <v>3.0000000000000001E-3</v>
+        <v>2.9616724738675002E-3</v>
       </c>
       <c r="N6">
-        <v>0.16300000000000001</v>
+        <v>0.16318718544328201</v>
       </c>
       <c r="O6">
-        <v>8.9999999999999993E-3</v>
+        <v>8.5232667040079004E-3</v>
       </c>
     </row>
     <row r="7" spans="1:15" x14ac:dyDescent="0.35">
@@ -1200,46 +1185,46 @@
         <v>14</v>
       </c>
       <c r="B7">
-        <v>0.60199999999999998</v>
+        <v>0.60210727178369605</v>
       </c>
       <c r="C7">
-        <v>0.54300000000000004</v>
+        <v>0.54307583180799901</v>
       </c>
       <c r="D7">
-        <v>0.77900000000000003</v>
+        <v>0.77938095238095195</v>
       </c>
       <c r="E7">
-        <v>0.50900000000000001</v>
+        <v>0.50904761904761897</v>
       </c>
       <c r="F7">
-        <v>0.19900000000000001</v>
+        <v>0.198888888888888</v>
       </c>
       <c r="G7">
-        <v>0.67100000000000004</v>
+        <v>0.671190476190476</v>
       </c>
       <c r="H7">
-        <v>6.5000000000000002E-2</v>
+        <v>6.5189711576832995E-2</v>
       </c>
       <c r="I7">
-        <v>0.27700000000000002</v>
+        <v>0.27706675453456098</v>
       </c>
       <c r="J7">
-        <v>6.0999999999999999E-2</v>
+        <v>6.0728637190243802E-2</v>
       </c>
       <c r="K7">
-        <v>0.215</v>
+        <v>0.215239063104916</v>
       </c>
       <c r="L7">
-        <v>0.189</v>
+        <v>0.18878242353852101</v>
       </c>
       <c r="M7">
-        <v>4.0000000000000001E-3</v>
+        <v>3.6585365853658001E-3</v>
       </c>
       <c r="N7">
-        <v>0.129</v>
+        <v>0.12945218737901601</v>
       </c>
       <c r="O7">
-        <v>8.0000000000000002E-3</v>
+        <v>7.5148496014933999E-3</v>
       </c>
     </row>
     <row r="8" spans="1:15" x14ac:dyDescent="0.35">
@@ -1247,46 +1232,46 @@
         <v>15</v>
       </c>
       <c r="B8">
-        <v>0.64400000000000002</v>
+        <v>0.64358388558528601</v>
       </c>
       <c r="C8">
-        <v>0.57999999999999996</v>
+        <v>0.58046835097600002</v>
       </c>
       <c r="D8">
-        <v>0.80900000000000005</v>
+        <v>0.80866666666666598</v>
       </c>
       <c r="E8">
-        <v>0.499</v>
+        <v>0.49880158730158702</v>
       </c>
       <c r="F8">
-        <v>0.17599999999999999</v>
+        <v>0.176023809523809</v>
       </c>
       <c r="G8">
-        <v>0.66200000000000003</v>
+        <v>0.66166666666666596</v>
       </c>
       <c r="H8">
-        <v>7.0000000000000007E-2</v>
+        <v>6.9811969717975805E-2</v>
       </c>
       <c r="I8">
-        <v>0.28799999999999998</v>
+        <v>0.288493429149345</v>
       </c>
       <c r="J8">
-        <v>6.3E-2</v>
+        <v>6.3078015375609697E-2</v>
       </c>
       <c r="K8">
-        <v>0.20799999999999999</v>
+        <v>0.208415602013162</v>
       </c>
       <c r="L8">
-        <v>0.17799999999999999</v>
+        <v>0.17799554781262</v>
       </c>
       <c r="M8">
-        <v>3.0000000000000001E-3</v>
+        <v>3.2520325203252002E-3</v>
       </c>
       <c r="N8">
-        <v>0.114</v>
+        <v>0.11410665892373199</v>
       </c>
       <c r="O8">
-        <v>8.0000000000000002E-3</v>
+        <v>7.7341084410785001E-3</v>
       </c>
     </row>
     <row r="9" spans="1:15" x14ac:dyDescent="0.35">
@@ -1298,180 +1283,50 @@
       <c r="A10" t="s">
         <v>17</v>
       </c>
+      <c r="B10">
+        <v>0.119829785492508</v>
+      </c>
+      <c r="C10">
+        <v>0.105115242495999</v>
+      </c>
+      <c r="D10">
+        <v>0.21572222222222201</v>
+      </c>
+      <c r="E10">
+        <v>6.1904761904760996E-3</v>
+      </c>
+      <c r="F10">
+        <v>5.0222222222222203E-2</v>
+      </c>
+      <c r="G10">
+        <v>0.18572222222222201</v>
+      </c>
+      <c r="H10">
+        <v>4.2522361588515998E-3</v>
+      </c>
+      <c r="I10">
+        <v>0.14271538296755101</v>
+      </c>
+      <c r="J10">
+        <v>3.07633226926829E-2</v>
+      </c>
+      <c r="K10">
+        <v>9.9980642663569402E-2</v>
+      </c>
+      <c r="L10">
+        <v>3.59417344173441E-2</v>
+      </c>
+      <c r="M10">
+        <v>1.3550135501355001E-3</v>
+      </c>
+      <c r="N10">
+        <v>6.9986449864498604E-2</v>
+      </c>
+      <c r="O10">
+        <v>1.5964415068753001E-3</v>
+      </c>
     </row>
   </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="B1:H1"/>
-    <mergeCell ref="I1:O1"/>
-  </mergeCells>
-  <conditionalFormatting sqref="B3:B8">
-    <cfRule type="colorScale" priority="14">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFCFCFF"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C3:C8">
-    <cfRule type="colorScale" priority="13">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFCFCFF"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D3:D8">
-    <cfRule type="colorScale" priority="12">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFCFCFF"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="E3:E8">
-    <cfRule type="colorScale" priority="11">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFCFCFF"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="F3:F8">
-    <cfRule type="colorScale" priority="10">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFCFCFF"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G3:G8">
-    <cfRule type="colorScale" priority="9">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFCFCFF"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H3:H8">
-    <cfRule type="colorScale" priority="8">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFCFCFF"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="I3:I8">
-    <cfRule type="colorScale" priority="7">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFCFCFF"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="J3:J8">
-    <cfRule type="colorScale" priority="6">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFCFCFF"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="K3:K8">
-    <cfRule type="colorScale" priority="5">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFCFCFF"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="L3:L8">
-    <cfRule type="colorScale" priority="4">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFCFCFF"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="M3:M8">
-    <cfRule type="colorScale" priority="3">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFCFCFF"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="N3:N8">
-    <cfRule type="colorScale" priority="2">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFCFCFF"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="O3:O8">
-    <cfRule type="colorScale" priority="1">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFCFCFF"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>